<commit_message>
Fix header formatting on Instructions tab
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator.xlsx
+++ b/Estimated_Tax_Calculator.xlsx
@@ -615,7 +615,7 @@
       <c r="A3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Quick Start Guide</t>
         </is>
@@ -643,7 +643,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Step 4: (Optional) Enter your estimated 'Itemized Deductions' if you expect to exceed the Standard Deduction.</t>
         </is>
@@ -660,7 +660,7 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Important Notes</t>
         </is>

</xml_diff>

<commit_message>
Fix: Excel structural shifting and dynamic array indexing; Add CA MFS support
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator.xlsx
+++ b/Estimated_Tax_Calculator.xlsx
@@ -281,6 +281,11 @@
     <comment ref="I33" authorId="0" shapeId="0">
       <text>
         <t>Warns if Head of Household is selected with zero dependents (legal but rare).</t>
+      </text>
+    </comment>
+    <comment ref="I34" authorId="0" shapeId="0">
+      <text>
+        <t>Flags if you have stale records from previous quarters which will artificially warp your pro-ration math.</t>
       </text>
     </comment>
   </commentList>
@@ -1079,7 +1084,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!B:B) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
+        <f>IF(MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0")=0, 0, (SUM('Wage Snapshots'!C:C) / MAX(1, MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0") - DATE(B8,1,1))) * (DATE(B8,12,31) - MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0")))</f>
         <v/>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -1096,7 +1101,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!C:D) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
+        <f>IF(MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0")=0, 0, (SUM('Wage Snapshots'!D:E) / MAX(1, MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0") - DATE(B8,1,1))) * (DATE(B8,12,31) - MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0")))</f>
         <v/>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -1170,7 +1175,7 @@
         </is>
       </c>
       <c r="B20" s="15">
-        <f>SUM('Wage Snapshots'!B:B) + (B15 * B14) + B13</f>
+        <f>SUM('Wage Snapshots'!C:C) + (B15 * B14) + B13</f>
         <v/>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -1191,7 +1196,7 @@
         </is>
       </c>
       <c r="B21" s="15">
-        <f>B20 - SUM('Wage Snapshots'!C:D) - (B16 * B14)</f>
+        <f>B20 - SUM('Wage Snapshots'!D:E) - (B16 * B14)</f>
         <v/>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -1212,7 +1217,7 @@
         </is>
       </c>
       <c r="B22" s="15">
-        <f>B20 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B16 * B14</f>
+        <f>B20 - SUM('Wage Snapshots'!D:D) - (SUM('Wage Snapshots'!D:D)/MAX(1, SUM('Wage Snapshots'!D:E))) * B16 * B14</f>
         <v/>
       </c>
       <c r="D22" s="2" t="n"/>
@@ -1307,7 +1312,7 @@
         </is>
       </c>
       <c r="J27">
-        <f>IF(OR(MAX('Wage Snapshots'!A:A)=0, (B9 - MAX('Wage Snapshots'!A:A)) &gt; 30), "🔴 !!! 30+ DAYS OLD !!!", "OK")</f>
+        <f>IF(OR(MAX('Wage Snapshots'!B:B)=0, (B9 - MAX('Wage Snapshots'!B:B)) &gt; 30), "🔴 !!! 30+ DAYS OLD !!!", "OK")</f>
         <v/>
       </c>
     </row>
@@ -1346,7 +1351,7 @@
         </is>
       </c>
       <c r="J29">
-        <f>IF(SUM('Wage Snapshots'!D:D)=0, "✅ No HSA Detected", IF(B22=B21, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
+        <f>IF(SUM('Wage Snapshots'!E:E)=0, "✅ No HSA Detected", IF(B22=B21, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
         <v/>
       </c>
     </row>
@@ -1435,7 +1440,15 @@
       </c>
       <c r="B34" s="15" t="n"/>
       <c r="D34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Stale Income Data:</t>
+        </is>
+      </c>
+      <c r="J34">
+        <f>IF(AND(MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0")&gt;0, ROUNDUP(MONTH(MINIFS('Wage Snapshots'!B:B, 'Wage Snapshots'!B:B, "&gt;0"))/3, 0) &lt; B10), "⚠️ WAGES FROM PRIOR QTR", IF(OR(AND(B10&gt;1, COUNTIF('Investment Income Snapshots'!A:A, "*Q1*")&gt;0), AND(B10&gt;2, COUNTIF('Investment Income Snapshots'!A:A, "*Q2*")&gt;0), AND(B10&gt;3, COUNTIF('Investment Income Snapshots'!A:A, "*Q3*")&gt;0)), "⚠️ INV. INCOME FROM PRIOR QTR", "OK"))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1645,7 +1658,7 @@
         </is>
       </c>
       <c r="B52" s="15">
-        <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
+        <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
       <c r="D52" s="2" t="n"/>
@@ -1671,7 +1684,7 @@
         </is>
       </c>
       <c r="B54" s="15">
-        <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
+        <f>SUM('Wage Snapshots'!G:G) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
         <v/>
       </c>
       <c r="D54" s="2" t="n"/>
@@ -1922,52 +1935,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Employer / Source</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Gross W-2 Income</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Pre-tax Deductions</t>
+          <t>Gross W-2 Income (YTD)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>HSA Contributions</t>
+          <t>Pre-tax Deductions (YTD)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Fed Tax Withheld</t>
+          <t>HSA Contributions (YTD)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CA Tax Withheld</t>
+          <t>Fed Tax Withheld (YTD)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>FICA/Med/SDI</t>
+          <t>CA Tax Withheld (YTD)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>FICA/Med/SDI (YTD)</t>
         </is>
       </c>
     </row>
@@ -1983,7 +2002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3154,7 +3173,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -3167,7 +3186,7 @@
         <v>0.01</v>
       </c>
       <c r="F58" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G58" t="n">
         <v>1000000</v>
@@ -3179,20 +3198,20 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>22158</v>
+        <v>11079</v>
       </c>
       <c r="D59" t="n">
-        <v>221.58</v>
+        <v>110.79</v>
       </c>
       <c r="E59" t="n">
         <v>0.02</v>
       </c>
       <c r="F59" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G59" t="n">
         <v>1000000</v>
@@ -3204,20 +3223,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>52528</v>
+        <v>26264</v>
       </c>
       <c r="D60" t="n">
-        <v>828.98</v>
+        <v>414.49</v>
       </c>
       <c r="E60" t="n">
         <v>0.04</v>
       </c>
       <c r="F60" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G60" t="n">
         <v>1000000</v>
@@ -3229,20 +3248,20 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>82904</v>
+        <v>41452</v>
       </c>
       <c r="D61" t="n">
-        <v>2044.02</v>
+        <v>1022.01</v>
       </c>
       <c r="E61" t="n">
         <v>0.06</v>
       </c>
       <c r="F61" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G61" t="n">
         <v>1000000</v>
@@ -3254,20 +3273,20 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>115084</v>
+        <v>57542</v>
       </c>
       <c r="D62" t="n">
-        <v>3974.82</v>
+        <v>1987.41</v>
       </c>
       <c r="E62" t="n">
         <v>0.08</v>
       </c>
       <c r="F62" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G62" t="n">
         <v>1000000</v>
@@ -3279,20 +3298,20 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>145448</v>
+        <v>72724</v>
       </c>
       <c r="D63" t="n">
-        <v>6403.94</v>
+        <v>3201.97</v>
       </c>
       <c r="E63" t="n">
         <v>0.093</v>
       </c>
       <c r="F63" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G63" t="n">
         <v>1000000</v>
@@ -3304,20 +3323,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>742958</v>
+        <v>371479</v>
       </c>
       <c r="D64" t="n">
-        <v>61972.37</v>
+        <v>31036.19</v>
       </c>
       <c r="E64" t="n">
         <v>0.103</v>
       </c>
       <c r="F64" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G64" t="n">
         <v>1000000</v>
@@ -3329,20 +3348,20 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>891542</v>
+        <v>445771</v>
       </c>
       <c r="D65" t="n">
-        <v>77276.52</v>
+        <v>38688.19</v>
       </c>
       <c r="E65" t="n">
         <v>0.113</v>
       </c>
       <c r="F65" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G65" t="n">
         <v>1000000</v>
@@ -3354,20 +3373,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1485906</v>
+        <v>742953</v>
       </c>
       <c r="D66" t="n">
-        <v>144439.65</v>
+        <v>72269.75</v>
       </c>
       <c r="E66" t="n">
         <v>0.123</v>
       </c>
       <c r="F66" t="n">
-        <v>11412</v>
+        <v>5706</v>
       </c>
       <c r="G66" t="n">
         <v>1000000</v>
@@ -3379,7 +3398,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -3404,14 +3423,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>22173</v>
+        <v>22158</v>
       </c>
       <c r="D68" t="n">
-        <v>221.73</v>
+        <v>221.58</v>
       </c>
       <c r="E68" t="n">
         <v>0.02</v>
@@ -3429,14 +3448,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>52530</v>
+        <v>52528</v>
       </c>
       <c r="D69" t="n">
-        <v>828.87</v>
+        <v>828.98</v>
       </c>
       <c r="E69" t="n">
         <v>0.04</v>
@@ -3454,14 +3473,14 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67716</v>
+        <v>82904</v>
       </c>
       <c r="D70" t="n">
-        <v>1436.31</v>
+        <v>2044.02</v>
       </c>
       <c r="E70" t="n">
         <v>0.06</v>
@@ -3479,14 +3498,14 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>83804</v>
+        <v>115084</v>
       </c>
       <c r="D71" t="n">
-        <v>2401.59</v>
+        <v>3974.82</v>
       </c>
       <c r="E71" t="n">
         <v>0.08</v>
@@ -3504,14 +3523,14 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>98990</v>
+        <v>145448</v>
       </c>
       <c r="D72" t="n">
-        <v>3616.47</v>
+        <v>6403.94</v>
       </c>
       <c r="E72" t="n">
         <v>0.093</v>
@@ -3529,14 +3548,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>505208</v>
+        <v>742958</v>
       </c>
       <c r="D73" t="n">
-        <v>41394.74</v>
+        <v>61972.37</v>
       </c>
       <c r="E73" t="n">
         <v>0.103</v>
@@ -3554,14 +3573,14 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>606251</v>
+        <v>891542</v>
       </c>
       <c r="D74" t="n">
-        <v>51802.17</v>
+        <v>77276.52</v>
       </c>
       <c r="E74" t="n">
         <v>0.113</v>
@@ -3579,14 +3598,14 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>HoH</t>
+          <t>MFJ</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1010417</v>
+        <v>1485906</v>
       </c>
       <c r="D75" t="n">
-        <v>97472.92999999999</v>
+        <v>144439.65</v>
       </c>
       <c r="E75" t="n">
         <v>0.123</v>
@@ -3598,39 +3617,79 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="76"/>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>HoH</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F76" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Table D: Surtaxes &amp; Phaseouts</t>
-        </is>
+      <c r="A77" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>HoH</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>22173</v>
+      </c>
+      <c r="D77" t="n">
+        <v>221.73</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F77" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G77" t="n">
+        <v>1000000</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
+      <c r="A78" t="n">
+        <v>2025</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>NIIT Threshold</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Addl Medicare</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>CTC Phaseout Start</t>
-        </is>
+          <t>HoH</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>52530</v>
+      </c>
+      <c r="D78" t="n">
+        <v>828.87</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F78" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1000000</v>
       </c>
     </row>
     <row r="79">
@@ -3639,17 +3698,23 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>HoH</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>200000</v>
+        <v>67716</v>
       </c>
       <c r="D79" t="n">
-        <v>200000</v>
+        <v>1436.31</v>
       </c>
       <c r="E79" t="n">
-        <v>200000</v>
+        <v>0.06</v>
+      </c>
+      <c r="F79" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G79" t="n">
+        <v>1000000</v>
       </c>
     </row>
     <row r="80">
@@ -3658,17 +3723,23 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MFJ</t>
+          <t>HoH</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>250000</v>
+        <v>83804</v>
       </c>
       <c r="D80" t="n">
-        <v>250000</v>
+        <v>2401.59</v>
       </c>
       <c r="E80" t="n">
-        <v>400000</v>
+        <v>0.08</v>
+      </c>
+      <c r="F80" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G80" t="n">
+        <v>1000000</v>
       </c>
     </row>
     <row r="81">
@@ -3677,17 +3748,23 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MFS</t>
+          <t>HoH</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>125000</v>
+        <v>98990</v>
       </c>
       <c r="D81" t="n">
-        <v>125000</v>
+        <v>3616.47</v>
       </c>
       <c r="E81" t="n">
-        <v>200000</v>
+        <v>0.093</v>
+      </c>
+      <c r="F81" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G81" t="n">
+        <v>1000000</v>
       </c>
     </row>
     <row r="82">
@@ -3700,12 +3777,179 @@
         </is>
       </c>
       <c r="C82" t="n">
+        <v>505208</v>
+      </c>
+      <c r="D82" t="n">
+        <v>41394.74</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="F82" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G82" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HoH</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>606251</v>
+      </c>
+      <c r="D83" t="n">
+        <v>51802.17</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="F83" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G83" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HoH</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>1010417</v>
+      </c>
+      <c r="D84" t="n">
+        <v>97472.92999999999</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="F84" t="n">
+        <v>11412</v>
+      </c>
+      <c r="G84" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="85"/>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Table D: Surtaxes &amp; Phaseouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>NIIT Threshold</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Addl Medicare</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>CTC Phaseout Start</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
         <v>200000</v>
       </c>
-      <c r="D82" t="n">
+      <c r="D88" t="n">
         <v>200000</v>
       </c>
-      <c r="E82" t="n">
+      <c r="E88" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MFJ</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D89" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E89" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MFS</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>125000</v>
+      </c>
+      <c r="D90" t="n">
+        <v>125000</v>
+      </c>
+      <c r="E90" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HoH</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D91" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E91" t="n">
         <v>200000</v>
       </c>
     </row>
@@ -3758,9 +4002,10 @@
 ---
 # Schema 1: Wage Snapshots (Paystubs)
 If the document is a paystub, RSU release confirmation, or W-2 income event, extract the data into the following columns exactly as defined:
-| Date | Gross W-2 Income | Pre-tax Deductions | HSA Contributions | Fed Tax Withheld | CA Tax Withheld | FICA/Med/SDI |
+| Employer / Source | Date | Gross W-2 Income | Pre-tax Deductions | HSA Contributions | Fed Tax Withheld | CA Tax Withheld | FICA/Med/SDI |
 |---|---|---|---|---|---|---|
 **Extraction Logic for Wage Snapshots:**
+*   **Employer / Source**: The name of the employer or source of income (e.g., `Google`, `Acme Corp`, `Spouse W-2`). If not clearly inferrable from the document, leave this field blank.
 *   **Date**: The date of the paystub or vest event (Format: MM/DD/YYYY).
 *   **Gross W-2 Income**: The **Year-to-Date (YTD)** gross pay, combining base salary, bonus payout, and/or the total taxable value of RSU vests up to this date.
 *   **Pre-tax Deductions**: The sum of all **YTD** pre-tax deductions (e.g., Traditional 401k, FSA, Health/Dental/Vision premiums). **CRITICAL IMPERATIVE**: Do **not** include HSA contributions in this sum.

</xml_diff>